<commit_message>
feat(data): update student records in CSV and modify Excel file for consistency
</commit_message>
<xml_diff>
--- a/sample_students.xlsx
+++ b/sample_students.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Enrollments" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,216 +398,255 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:O3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Student Ref</v>
+      </c>
+      <c r="B1" t="str">
         <v>Name (English)</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Name (Urdu)</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Father Name</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Phone Number</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Is Minor</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Guardian Name</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Guardian Phone</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Gender</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Date of Birth</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Marital Status</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Qualification</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Occupation</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Address</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Profile Picture</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Muhammad Usman</v>
+        <v>S1</v>
       </c>
       <c r="B2" t="str">
-        <v>محمد عثمان</v>
+        <v>Ahmad Raza</v>
       </c>
       <c r="C2" t="str">
-        <v>Tariq Mahmood</v>
+        <v>احمد رضا</v>
       </c>
       <c r="D2" t="str">
+        <v>Muhammad Ali</v>
+      </c>
+      <c r="E2" t="str">
         <v>03001234567</v>
       </c>
-      <c r="E2" t="str">
-        <v>No</v>
-      </c>
       <c r="F2" t="str">
-        <v/>
+        <v>false</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>male</v>
       </c>
-      <c r="I2" t="str">
-        <v>1996-04-12</v>
-      </c>
       <c r="J2" t="str">
+        <v>05-15-1998</v>
+      </c>
+      <c r="K2" t="str">
         <v>Single</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Bachelors</v>
       </c>
-      <c r="L2" t="str">
-        <v>Software Engineer</v>
-      </c>
       <c r="M2" t="str">
-        <v>House # 12 Block B Lahore</v>
+        <v>Student</v>
+      </c>
+      <c r="N2" t="str">
+        <v>House 123, Block A</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://images.unsplash.com/photo-1535713875002-d1d0cf377fde</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Ayesha Bibi</v>
+        <v>S2</v>
       </c>
       <c r="B3" t="str">
-        <v>عائشہ بی بی</v>
+        <v>Fatima Ali</v>
       </c>
       <c r="C3" t="str">
-        <v>Muhammad Akhtar</v>
+        <v>فاطمہ علی</v>
       </c>
       <c r="D3" t="str">
-        <v>03019876543</v>
+        <v>Ali Hassan</v>
       </c>
       <c r="E3" t="str">
-        <v>No</v>
+        <v/>
       </c>
       <c r="F3" t="str">
+        <v>true</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Ali Hassan</v>
+      </c>
+      <c r="H3" t="str">
+        <v>03009876543</v>
+      </c>
+      <c r="I3" t="str">
+        <v>female</v>
+      </c>
+      <c r="J3" t="str">
+        <v>08-20-2015</v>
+      </c>
+      <c r="K3" t="str">
         <v/>
       </c>
+      <c r="L3" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Student</v>
+      </c>
+      <c r="N3" t="str">
+        <v>House 456, Block B</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://images.unsplash.com/photo-1494790108377-be9c29b29330</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Student Ref</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Class ID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Enrolled On</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Prior Level</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes (Urdu)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Amount Paid</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Payment Method</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>S1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>123e4567-e89b-12d3-a456-426614174000</v>
+      </c>
+      <c r="C2" t="str">
+        <v>01-15-2024</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Beginner</v>
+      </c>
+      <c r="E2" t="str">
+        <v>مبتدی طالب علم</v>
+      </c>
+      <c r="F2" t="str">
+        <v>5000</v>
+      </c>
+      <c r="G2" t="str">
+        <v>cash</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>S2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>123e4567-e89b-12d3-a456-426614174000</v>
+      </c>
+      <c r="C3" t="str">
+        <v>01-15-2024</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Nazra</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>3000</v>
+      </c>
       <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>female</v>
-      </c>
-      <c r="I3" t="str">
-        <v>2001-08-25</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Single</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Intermediate</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Student</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Flat 402 Paragon City Lahore</v>
+        <v>cash</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Zaid Ahmed</v>
+        <v>S2</v>
       </c>
       <c r="B4" t="str">
-        <v>زید احمد</v>
+        <v>987f6543-e21b-32d1-b654-987654321000</v>
       </c>
       <c r="C4" t="str">
-        <v>Bilal Ahmed</v>
+        <v>01-15-2024</v>
       </c>
       <c r="D4" t="str">
+        <v>Hifz Part 1</v>
+      </c>
+      <c r="E4" t="str">
         <v/>
       </c>
-      <c r="E4" t="str">
-        <v>Yes</v>
-      </c>
       <c r="F4" t="str">
-        <v>Bilal Ahmed</v>
+        <v>2000</v>
       </c>
       <c r="G4" t="str">
-        <v>03214567890</v>
-      </c>
-      <c r="H4" t="str">
-        <v>male</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2014-11-05</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Single</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Primary</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Student</v>
-      </c>
-      <c r="M4" t="str">
-        <v>House # 55 Sector C Johar Town</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Zainab Fatima</v>
-      </c>
-      <c r="B5" t="str">
-        <v>زینب فاطمہ</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Kamran Ali</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Kamran Ali</v>
-      </c>
-      <c r="G5" t="str">
-        <v>03338765432</v>
-      </c>
-      <c r="H5" t="str">
-        <v>female</v>
-      </c>
-      <c r="I5" t="str">
-        <v>2016-02-18</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Single</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Primary</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Student</v>
-      </c>
-      <c r="M5" t="str">
-        <v>House # 18 Model Town Lahore</v>
+        <v>online</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>